<commit_message>
Update all local changes
</commit_message>
<xml_diff>
--- a/IGR_Master/Data/Documents/Config.xlsx
+++ b/IGR_Master/Data/Documents/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DeokateLaxman\Documents\UiPathAutomation\IGR_Master\Data\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UiPath_GitProjects\IGR_Master\Data\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{206AC850-4067-4607-9229-85BA13D6C69A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{482A09D8-9158-4CD2-8E2B-6D2FE25705C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -360,7 +360,7 @@
     <t>AdPDetails</t>
   </si>
   <si>
-    <t>C:\Users\DeokateLaxman\Documents\UiPathAutomation\IGR_Master\Data\Documents</t>
+    <t>C:\UiPath_GitProjects\IGR_Master\Data\Documents</t>
   </si>
 </sst>
 </file>
@@ -710,12 +710,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z994"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.54296875" customWidth="1"/>
-    <col min="2" max="2" width="95.1796875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="81.453125" customWidth="1"/>
-    <col min="4" max="26" width="8.7265625" customWidth="1"/>
+    <col min="1" max="1" width="43.5703125" customWidth="1"/>
+    <col min="2" max="2" width="95.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="81.42578125" customWidth="1"/>
+    <col min="4" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -752,7 +752,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" s="4" customFormat="1" ht="15.5">
+    <row r="2" spans="1:26" s="4" customFormat="1" ht="15.75">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -760,7 +760,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="18.5">
+    <row r="3" spans="1:26" ht="18.75">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -2038,12 +2038,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.453125" customWidth="1"/>
-    <col min="4" max="26" width="8.7265625" customWidth="1"/>
+    <col min="3" max="3" width="75.42578125" customWidth="1"/>
+    <col min="4" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -2080,7 +2080,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="29">
+    <row r="2" spans="1:26" ht="30">
       <c r="A2" t="s">
         <v>71</v>
       </c>
@@ -2091,7 +2091,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="43.5">
+    <row r="3" spans="1:26" ht="45">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -2205,7 +2205,7 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="29">
+    <row r="17" spans="1:3" ht="45">
       <c r="A17" t="s">
         <v>100</v>
       </c>
@@ -3230,12 +3230,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.81640625" customWidth="1"/>
-    <col min="2" max="2" width="30.1796875" customWidth="1"/>
-    <col min="3" max="3" width="60.26953125" customWidth="1"/>
-    <col min="4" max="26" width="65.453125" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" customWidth="1"/>
+    <col min="3" max="3" width="60.28515625" customWidth="1"/>
+    <col min="4" max="26" width="65.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">

</xml_diff>